<commit_message>
new feature for nonLFF mapping. have to input ticket number in third column of pydump.
</commit_message>
<xml_diff>
--- a/Inputs/PyDump.xlsx
+++ b/Inputs/PyDump.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pierre\Downloads\GCOH\GCOHFilesTicketsEtc\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C0A93B-68D5-4B91-B8BD-B33C47A2A160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED31C3F6-8FC2-462D-9B62-9EABFDD26C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6A12B107-397F-4BA6-8F78-4BB99A484E33}"/>
+    <workbookView xWindow="8430" yWindow="4140" windowWidth="12060" windowHeight="13170" xr2:uid="{6A12B107-397F-4BA6-8F78-4BB99A484E33}"/>
   </bookViews>
   <sheets>
     <sheet name="Dump" sheetId="1" r:id="rId1"/>
@@ -19,21 +19,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Dump!$A$1:$B$1</definedName>
     <definedName name="ID" localSheetId="0" hidden="1">"caea3f49-dfad-4101-9423-d5e90b427b0f"</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -43,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="98">
   <si>
     <t>Object</t>
   </si>
@@ -331,6 +320,12 @@
   </si>
   <si>
     <t>CTEMPEU_1000CH70ADF100</t>
+  </si>
+  <si>
+    <t>Ticket</t>
+  </si>
+  <si>
+    <t>FR7558422</t>
   </si>
 </sst>
 </file>
@@ -743,7 +738,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -888,6 +883,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -968,8 +976,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="69">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1414,627 +1423,858 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9544D389-BCBF-4017-8282-1DF88DB28091}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:B77"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.5703125" customWidth="1"/>
     <col min="2" max="2" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
       <c r="B15" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
       <c r="B16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>24</v>
       </c>
       <c r="B17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>26</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>27</v>
       </c>
       <c r="B19" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>28</v>
       </c>
       <c r="B20" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>29</v>
       </c>
       <c r="B21" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>30</v>
       </c>
       <c r="B22" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>31</v>
       </c>
       <c r="B23" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>32</v>
       </c>
       <c r="B24" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>34</v>
       </c>
       <c r="B25" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>36</v>
       </c>
       <c r="B26" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>37</v>
       </c>
       <c r="B27" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>39</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C28" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
       <c r="B29" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>42</v>
       </c>
       <c r="B30" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C30" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>43</v>
       </c>
       <c r="B31" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>44</v>
       </c>
       <c r="B32" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>45</v>
       </c>
       <c r="B33" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>46</v>
       </c>
       <c r="B34" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C34" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>48</v>
       </c>
       <c r="B35" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C35" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>50</v>
       </c>
       <c r="B36" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C36" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>51</v>
       </c>
       <c r="B37" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C37" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>52</v>
       </c>
       <c r="B38" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C38" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>54</v>
       </c>
       <c r="B39" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C39" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>56</v>
       </c>
       <c r="B40" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C40" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>57</v>
       </c>
       <c r="B41" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C41" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>58</v>
       </c>
       <c r="B42" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C42" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>59</v>
       </c>
       <c r="B43" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C43" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>60</v>
       </c>
       <c r="B44" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C44" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>61</v>
       </c>
       <c r="B45" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C45" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>62</v>
       </c>
       <c r="B46" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C46" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>63</v>
       </c>
       <c r="B47" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C47" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>64</v>
       </c>
       <c r="B48" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C48" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>65</v>
       </c>
       <c r="B49" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C49" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>66</v>
       </c>
       <c r="B50" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C50" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>67</v>
       </c>
       <c r="B51" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C51" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>68</v>
       </c>
       <c r="B52" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C52" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>69</v>
       </c>
       <c r="B53" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C53" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>70</v>
       </c>
       <c r="B54" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C54" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>71</v>
       </c>
       <c r="B55" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C55" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>72</v>
       </c>
       <c r="B56" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C56" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>73</v>
       </c>
       <c r="B57" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C57" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>74</v>
       </c>
       <c r="B58" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C58" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>75</v>
       </c>
       <c r="B59" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C59" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>76</v>
       </c>
       <c r="B60" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C60" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>77</v>
       </c>
       <c r="B61" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C61" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>78</v>
       </c>
       <c r="B62" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C62" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>79</v>
       </c>
       <c r="B63" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C63" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>80</v>
       </c>
       <c r="B64" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C64" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>81</v>
       </c>
       <c r="B65" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C65" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>82</v>
       </c>
       <c r="B66" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C66" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>83</v>
       </c>
       <c r="B67" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C67" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>85</v>
       </c>
       <c r="B68" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C68" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>86</v>
       </c>
       <c r="B69" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C69" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>87</v>
       </c>
       <c r="B70" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C70" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>89</v>
       </c>
       <c r="B71" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C71" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>90</v>
       </c>
       <c r="B72" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C72" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>91</v>
       </c>
       <c r="B73" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C73" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>92</v>
       </c>
       <c r="B74" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C74" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>93</v>
       </c>
       <c r="B75" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C75" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>94</v>
       </c>
       <c r="B76" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C76" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>95</v>
       </c>
       <c r="B77" t="s">
         <v>88</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>